<commit_message>
WIP: auto-save — 1 file(s) — 2026-03-31 14:30 UTC —
</commit_message>
<xml_diff>
--- a/Scripture_Alive_Client_Report.xlsx
+++ b/Scripture_Alive_Client_Report.xlsx
@@ -7,11 +7,9 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scripture Alive Updates" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Task List" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Scripture Alive Updates'!$A$4:$E$25</definedName>
-  </definedNames>
+  <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -36,13 +34,13 @@
     <font>
       <name val="Arial"/>
       <color rgb="00666666"/>
-      <sz val="10"/>
+      <sz val="9"/>
     </font>
     <font>
       <name val="Arial"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="12"/>
+      <sz val="11"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -104,25 +102,19 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -498,27 +490,25 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E27"/>
+  <dimension ref="A1:C23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="28" customWidth="1" min="3" max="3"/>
-    <col width="65" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="75" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1">
+    <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Scripture Alive - Website Updates &amp; SEO Improvements</t>
+          <t>Scripture Alive — Revision Task List</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Completed: March 31, 2026 | Prepared by: Spirit Media Publishing</t>
+          <t>Date: March 31, 2026 | Prepared by: Spirit Media Publishing</t>
         </is>
       </c>
     </row>
@@ -530,20 +520,10 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Category</t>
+          <t>Task Description</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>Task</t>
-        </is>
-      </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>What Was Done</t>
-        </is>
-      </c>
-      <c r="E4" s="3" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
@@ -557,20 +537,10 @@
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>Design</t>
+          <t>Dancing Script font applied to every heading on all pages: Homepage (Making Scripture Unforgettable, Dedicated to Proclaiming, Pure Scripture, Skillfully Dramatized, Impacting Lives, Unique and Memorable), Events, Workshops, Guest Speaking, Videos, Interviews, Contact, Performances</t>
         </is>
       </c>
       <c r="C5" s="6" t="inlineStr">
-        <is>
-          <t>Dancing Script Typography</t>
-        </is>
-      </c>
-      <c r="D5" s="7" t="inlineStr">
-        <is>
-          <t>Applied Dancing Script (decorative cursive font) to all page headings across the entire site: Homepage, Events, Workshops, Guest Speaking, Videos, Interviews, Contact, and Performances pages.</t>
-        </is>
-      </c>
-      <c r="E5" s="8" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
@@ -584,20 +554,10 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Design</t>
+          <t>Events Page: Replaced "Upcoming Events" with "Events Calendar" (with s). New description from Event Calendar section. Date headings (April 2026) use regular font — NOT Dancing Script. Event descriptions added to Sanity (8/8 events) and shown in modal popup. Page reordered: 1) Events Calendar 2) Download booking info 3) Event listings 4) Performance/Workshop/Speaking cards 5) Interested in Booking Jeremy?</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
-        <is>
-          <t>Typography Cleanup</t>
-        </is>
-      </c>
-      <c r="D6" s="7" t="inlineStr">
-        <is>
-          <t>Reduced base font size from 18px to 16px for better readability. Event titles, card labels, and date headings use clean sans-serif font.</t>
-        </is>
-      </c>
-      <c r="E6" s="8" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
@@ -611,20 +571,10 @@
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>Events</t>
+          <t>Performances Page: Fixed mobile image cutoff — images now shrink to fit instead of cropping. Last section renamed from "Stories" to "Narratives".</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
-        <is>
-          <t>Page Restructured</t>
-        </is>
-      </c>
-      <c r="D7" s="7" t="inlineStr">
-        <is>
-          <t>Replaced "Upcoming Events" with "Events Calendar". Reordered: Events Calendar &gt; Download booking info &gt; Event listings &gt; Booking cards &gt; Interested in Booking Jeremy?</t>
-        </is>
-      </c>
-      <c r="E7" s="8" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
@@ -633,25 +583,15 @@
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3B</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Events</t>
+          <t>Accordion Pages: Fixed all missing/cut-off images. All 9 performances now have correct images from Sanity (Daniel, Johns Gospel, Sermon Starters, Paul, Elijah, Peter, One-Man Passion Play, The Advent Story, The Beginning and the End). Images display fully without cropping.</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
-        <is>
-          <t>Event Descriptions</t>
-        </is>
-      </c>
-      <c r="D8" s="7" t="inlineStr">
-        <is>
-          <t>Full descriptions added for all 8 upcoming events in the CMS. Shown in event detail modal with venue, date, map, calendar link, and share buttons.</t>
-        </is>
-      </c>
-      <c r="E8" s="8" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
@@ -660,25 +600,15 @@
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3C</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>Events</t>
+          <t>Sermon Starters: Added the official 4-panel poster image (Genesis, Job, Acts, Revelation) to the Books accordion page.</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
-        <is>
-          <t>Date Heading Fonts</t>
-        </is>
-      </c>
-      <c r="D9" s="7" t="inlineStr">
-        <is>
-          <t>Month headings ("April 2026") now use clean Roboto Slab font instead of decorative script for readability.</t>
-        </is>
-      </c>
-      <c r="E9" s="8" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
@@ -687,25 +617,15 @@
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>4</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>Performances</t>
+          <t>Guest Speaking Page: Replaced all 6 mixed-up images with the correct original artwork from the current live WordPress site (Elijah, Daniel, Paul, Johns Gospel, 1 Peter, Custom Programs).</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
-        <is>
-          <t>Mobile Image Fix</t>
-        </is>
-      </c>
-      <c r="D10" s="7" t="inlineStr">
-        <is>
-          <t>Performance tile images no longer crop on mobile. Images shrink to fit while showing the full artwork.</t>
-        </is>
-      </c>
-      <c r="E10" s="8" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
@@ -714,25 +634,15 @@
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Performances</t>
+          <t>Store Page: Replaced podcast studio photo with the correct "No More Excuses — Power Tools for Scripture Memory" banner from the current site. Centered layout with padding.</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
-        <is>
-          <t>Stories to Narratives</t>
-        </is>
-      </c>
-      <c r="D11" s="7" t="inlineStr">
-        <is>
-          <t>Renamed third performance category from "Stories" to "Narratives" across all pages and SEO metadata.</t>
-        </is>
-      </c>
-      <c r="E11" s="8" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
@@ -741,25 +651,15 @@
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>6</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>Performances</t>
+          <t>Videos Page: Redesigned from large single videos to 3-column grid. Two sections: Performance Samples (5 Vimeo clips) and Full Performances on YouTube (6 videos). Added "See YouTube Channel for More" button.</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
-        <is>
-          <t>Accordion Page Images</t>
-        </is>
-      </c>
-      <c r="D12" s="7" t="inlineStr">
-        <is>
-          <t>Added correct images for all 9 performances on accordion detail pages. No more missing or placeholder images.</t>
-        </is>
-      </c>
-      <c r="E12" s="8" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
@@ -768,25 +668,15 @@
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>Performances</t>
+          <t>Resources Header Button: /resources page is now hidden (direct URL access only). Nav "Resources" is a dropdown trigger for Store, Videos, Interviews, Blog — does not link to /resources.</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
-        <is>
-          <t>Sermon Starters Image</t>
-        </is>
-      </c>
-      <c r="D13" s="7" t="inlineStr">
-        <is>
-          <t>Added official Sermon Starters poster (Genesis/Job/Acts/Revelation 4-panel collage) to the Books accordion page.</t>
-        </is>
-      </c>
-      <c r="E13" s="8" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
@@ -795,25 +685,15 @@
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>8</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>Guest Speaking</t>
+          <t>Book Jeremy Button: Fixed disfigured desktop layout. Responsive sizing, no text wrapping. Nav breakpoint adjusted from md to lg to fit all 8 nav items.</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr">
-        <is>
-          <t>Fixed Wrong Images</t>
-        </is>
-      </c>
-      <c r="D14" s="7" t="inlineStr">
-        <is>
-          <t>Replaced incorrect images for all 6 speaking topics with original artwork from the current live site.</t>
-        </is>
-      </c>
-      <c r="E14" s="8" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
@@ -822,25 +702,15 @@
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>Store</t>
+          <t>Workshops Accordion Pages: Created 3 new sub-pages matching the Performances structure — Foundations Track (How to Memorize Scripture for Life, Speaking Gods Word with Confidence, How to Study the Bible for Yourself), Discipleship Track (Praying the Word, Witnessing with the Word, Holding Fast to Gods Word), Advanced Track (Acting the Word). Main workshops page updated to show all 3 tracks with image tiles.</t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
-        <is>
-          <t>Hero Banner Updated</t>
-        </is>
-      </c>
-      <c r="D15" s="7" t="inlineStr">
-        <is>
-          <t>Replaced incorrect photo with the official "No More Excuses - Power Tools for Scripture Memory" banner.</t>
-        </is>
-      </c>
-      <c r="E15" s="8" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
@@ -849,25 +719,15 @@
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>SEO 1</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>Videos</t>
+          <t>Hero button changed to single "Book Jeremy" CTA. /book-jeremy page now has service options + 2 endorsement quotes + booking inquiry form — full conversion path on one page.</t>
         </is>
       </c>
       <c r="C16" s="6" t="inlineStr">
-        <is>
-          <t>Redesigned Layout</t>
-        </is>
-      </c>
-      <c r="D16" s="7" t="inlineStr">
-        <is>
-          <t>3-column grid layout. Two sections: Performance Samples (5 Vimeo) and Full Performances on YouTube (6 videos). Added "See YouTube Channel for More" button.</t>
-        </is>
-      </c>
-      <c r="E16" s="8" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
@@ -876,25 +736,15 @@
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>SEO 2</t>
         </is>
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Endorsement/social proof section added to homepage directly before the service tiles with testimonial quote, attribution, and "Read More Endorsements" link.</t>
         </is>
       </c>
       <c r="C17" s="6" t="inlineStr">
-        <is>
-          <t>Resources Hidden</t>
-        </is>
-      </c>
-      <c r="D17" s="7" t="inlineStr">
-        <is>
-          <t>/resources page accessible only via direct URL. Nav dropdown shows Store, Videos, Interviews, Blog.</t>
-        </is>
-      </c>
-      <c r="E17" s="8" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
@@ -903,25 +753,15 @@
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>14</t>
+          <t>SEO 3</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Navigation rebuilt to 8 items: Home | Performances | Workshops | Speaking | Endorsements | Resources (Dropdown: Store, Videos, Interviews, Blog) | Events | Book Jeremy (button)</t>
         </is>
       </c>
       <c r="C18" s="6" t="inlineStr">
-        <is>
-          <t>Book Jeremy Button</t>
-        </is>
-      </c>
-      <c r="D18" s="7" t="inlineStr">
-        <is>
-          <t>Fixed disfigured desktop button. Responsive sizing, no text wrapping. Nav breakpoint adjusted for 8 items.</t>
-        </is>
-      </c>
-      <c r="E18" s="8" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
@@ -930,25 +770,15 @@
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>SEO 4</t>
         </is>
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>Navigation</t>
+          <t>Service tile labels added to homepage — each tile now shows title + one-line description overlay: Scripture Performances, Bible Memory Workshops, Guest Speaking. Visible on mobile without hovering.</t>
         </is>
       </c>
       <c r="C19" s="6" t="inlineStr">
-        <is>
-          <t>New 8-Item Nav</t>
-        </is>
-      </c>
-      <c r="D19" s="7" t="inlineStr">
-        <is>
-          <t>Home | Performances | Workshops | Speaking | Endorsements | Resources (dropdown) | Events | Book Jeremy (button)</t>
-        </is>
-      </c>
-      <c r="E19" s="8" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
@@ -957,25 +787,15 @@
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>SEO 5</t>
         </is>
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>Workshops</t>
+          <t>Refer Jeremy button removed from hero. Single "Book Jeremy" CTA. Cleaner conversion path for decision-makers.</t>
         </is>
       </c>
       <c r="C20" s="6" t="inlineStr">
-        <is>
-          <t>Accordion Sub-Pages</t>
-        </is>
-      </c>
-      <c r="D20" s="7" t="inlineStr">
-        <is>
-          <t>Created 3 new workshop track pages: Foundations (3 workshops), Discipleship (3 workshops), Advanced (1 workshop). Each with accordion cards, images, descriptions, and booking buttons.</t>
-        </is>
-      </c>
-      <c r="E20" s="8" t="inlineStr">
         <is>
           <t>Complete</t>
         </is>
@@ -984,151 +804,32 @@
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>SEO 6</t>
         </is>
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>Homepage</t>
+          <t>Added audience qualifier below tagline: "Available for churches, conferences, camps, schools, and special events". Tagline and subtitle kept above it.</t>
         </is>
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
-          <t>Single Book Jeremy CTA</t>
-        </is>
-      </c>
-      <c r="D21" s="7" t="inlineStr">
-        <is>
-          <t>Replaced dual buttons (Invite + Refer) with single prominent "Book Jeremy" button for cleaner conversion.</t>
-        </is>
-      </c>
-      <c r="E21" s="8" t="inlineStr">
-        <is>
-          <t>Complete</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="4" t="inlineStr">
-        <is>
-          <t>18</t>
-        </is>
-      </c>
-      <c r="B22" s="5" t="inlineStr">
-        <is>
-          <t>Homepage</t>
-        </is>
-      </c>
-      <c r="C22" s="6" t="inlineStr">
-        <is>
-          <t>Social Proof Section</t>
-        </is>
-      </c>
-      <c r="D22" s="7" t="inlineStr">
-        <is>
-          <t>Added endorsement quote section before service tiles with testimonial attribution and "Read More Endorsements" link.</t>
-        </is>
-      </c>
-      <c r="E22" s="8" t="inlineStr">
-        <is>
           <t>Complete</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="4" t="inlineStr">
-        <is>
-          <t>19</t>
-        </is>
-      </c>
-      <c r="B23" s="5" t="inlineStr">
-        <is>
-          <t>Homepage</t>
-        </is>
-      </c>
-      <c r="C23" s="6" t="inlineStr">
-        <is>
-          <t>Service Tile Labels</t>
-        </is>
-      </c>
-      <c r="D23" s="7" t="inlineStr">
-        <is>
-          <t>Added title + description overlay to 3 service tiles: Scripture Performances, Bible Memory Workshops, Guest Speaking. Visible on mobile without hovering.</t>
-        </is>
-      </c>
-      <c r="E23" s="8" t="inlineStr">
-        <is>
-          <t>Complete</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="4" t="inlineStr">
-        <is>
-          <t>20</t>
-        </is>
-      </c>
-      <c r="B24" s="5" t="inlineStr">
-        <is>
-          <t>Homepage</t>
-        </is>
-      </c>
-      <c r="C24" s="6" t="inlineStr">
-        <is>
-          <t>Audience Qualifier</t>
-        </is>
-      </c>
-      <c r="D24" s="7" t="inlineStr">
-        <is>
-          <t>Added "Available for churches, conferences, camps, schools, and special events" below the tagline.</t>
-        </is>
-      </c>
-      <c r="E24" s="8" t="inlineStr">
-        <is>
-          <t>Complete</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="4" t="inlineStr">
-        <is>
-          <t>21</t>
-        </is>
-      </c>
-      <c r="B25" s="5" t="inlineStr">
-        <is>
-          <t>Booking</t>
-        </is>
-      </c>
-      <c r="C25" s="6" t="inlineStr">
-        <is>
-          <t>Endorsements Added</t>
-        </is>
-      </c>
-      <c r="D25" s="7" t="inlineStr">
-        <is>
-          <t>Added 2 endorsement quotes from church leaders to /book-jeremy page. Full conversion path: service options &gt; social proof &gt; inquiry form.</t>
-        </is>
-      </c>
-      <c r="E25" s="8" t="inlineStr">
-        <is>
-          <t>Complete</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="9" t="inlineStr">
-        <is>
-          <t>Total: 21 tasks completed. All changes on dev branch pending client review before going live.</t>
+      <c r="A23" s="7" t="inlineStr">
+        <is>
+          <t>Total: 17 tasks — All Complete. Changes on dev branch pending review before going live.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:E25"/>
   <mergeCells count="3">
-    <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A27:E27"/>
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A23:C23"/>
+    <mergeCell ref="A2:C2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>